<commit_message>
Cronograma: anadir la tarea 79, seleccion de foco en mi_prueba_dlhm y el modelo de Lopera
Semana 11, fase F2, Hecho, con los commits 4e08e49050 (el arreglo de la ida
de CamposT/dlhm.py) y dfe6fe7a27 como evidencia. La nota lleva los numeros
medidos: el exacto a 3.0000 en las tres metricas a escala real, el de Carlos
a 2 um, el ~0.03 viejo explicado por la geometria de referencia_a_escala(),
y el modelo de Lopera enfocando +14 a +20 um fuera de Z_REAL por su nucleo
paraxial.

Solo cambian las 9 celdas de la fila 82 y el autofiltro, que pasa a A3:I82;
los IDs siguen de 1 a 79 sin huecos, cada uno en su fila N+3. La tarea 77
(ROI y bloques de memoria en barrido_foco) sigue En curso: su codigo no esta
commiteado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Cronograma_TG_DLHM.xlsx
+++ b/docs/Cronograma_TG_DLHM.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Hitos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tareas'!$A$3:$I$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tareas'!$A$3:$I$82</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -1314,7 +1314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" style="22" min="1" max="1"/>
@@ -4619,8 +4619,51 @@
         </is>
       </c>
     </row>
+    <row r="82" ht="25.5" customHeight="1" s="22">
+      <c r="A82" s="12" t="n">
+        <v>79</v>
+      </c>
+      <c r="B82" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C82" s="12" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="D82" s="13" t="inlineStr">
+        <is>
+          <t>Portar la seleccion de foco de barrido_foco a mi_prueba_dlhm (motores exacto y de Carlos) y anadir el modelo de Lopera como segundo simulador</t>
+        </is>
+      </c>
+      <c r="E82" s="13" t="inlineStr">
+        <is>
+          <t>scripts/mi_prueba_dlhm.py + tests/test_mi_prueba_dlhm_seleccion.py + arreglo de CamposT/dlhm.py</t>
+        </is>
+      </c>
+      <c r="F82" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G82" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H82" s="12" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="I82" s="13" t="inlineStr">
+        <is>
+          <t>Commits 4e08e49050 (CamposT/dlhm.py) y dfe6fe7a27. mi_prueba_dlhm.py elige el foco con los parametros de seleccion de barrido_foco (Tamura, Pearson y SSIM sobre la misma reconstruccion, grueso + fino, ROI o cuarto central, tabla, curvas.npz y dos figuras; metricas copiadas con prueba ast) y dos motores: exacto (CamposT.dlhm, holograma entero) y de Carlos (reconstruir() sobre el recorte: hay que dividir por |U0|^2 -0.84 frente a 0.21-, tomar la huella del 1/M central y usar un ROI cuadrado). BenchmarkTarget simulado 3000x4000 a z = 3 mm: exacto 3.0000 en las tres metricas, tambien con Z_REAL a medio paso de la rejilla; Carlos (ROI 1024) a 2 um; objeto de fase, -Tamura a 1 um. El ~0.03 del script viejo era la geometria de referencia_a_escala(): +0.051 frente a -0.731 con la huella. Arreglado de paso holograma() de CamposT/dlhm.py: el soporte recortaba la frecuencia del otro eje a 1/lambda y pedia 86.7 GB con 3000x4000; ahora 40 s en GPU y RS sigue en 3.7e-6. SIMULADOR = 'lopera': el modelo de Lopera et al. 2024 (su dlhm() copiada literal, verificada bit a bit contra su codigo): su holograma reconstruido exacto enfoca +14 a +20 um fuera de Z_REAL; sin Brown-Conrady, envolvente ni 8 bits sigue (+16 a +27 um): es su nucleo paraxial (contra la ida exacta, 1.00000 con objeto liso y 0.895 con detalle fino). 49 pruebas nuevas; suite 551 passed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:I81"/>
+  <autoFilter ref="A3:I82"/>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>

</xml_diff>